<commit_message>
Ajustar parcial Power BI con calendario propio
</commit_message>
<xml_diff>
--- a/clase_s1/datasets_powerbi_parcial/02_citas_clinica_powerbi.xlsx
+++ b/clase_s1/datasets_powerbi_parcial/02_citas_clinica_powerbi.xlsx
@@ -2,10 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Citas" sheetId="1" r:id="Rbf557dd927d74854"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pacientes" sheetId="2" r:id="Rfe6da811ea42493a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Medicos" sheetId="3" r:id="Refe8a1e260894d09"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Calendario" sheetId="4" r:id="R2e300b872ba44c89"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Citas" sheetId="1" r:id="R2694821280e542f3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pacientes" sheetId="2" r:id="R37ddee2912034ebf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Medicos" sheetId="3" r:id="Rd19d58e4775746ef"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -111,19 +110,6 @@
     <x:tableColumn id="1" name="MedicoID"/>
     <x:tableColumn id="2" name="Especialidad"/>
     <x:tableColumn id="3" name="Sede"/>
-  </x:tableColumns>
-  <x:tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
-</x:table>
-</file>
-
-<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="CalendarioClinica" displayName="CalendarioClinica" ref="A1:E121" headerRowCount="1">
-  <x:tableColumns count="5">
-    <x:tableColumn id="1" name="Fecha"/>
-    <x:tableColumn id="2" name="Anio"/>
-    <x:tableColumn id="3" name="MesNumero"/>
-    <x:tableColumn id="4" name="Mes"/>
-    <x:tableColumn id="5" name="TipoDia"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
 </x:table>
@@ -2631,7 +2617,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R325f238f597e4156"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R598d60da1c0349b2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2747,7 +2733,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R967c02c091b949b7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rba36adcce21b47c7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2819,2083 +2805,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8dccf7de5e0a43e6"/>
-  </x:tableParts>
-</x:worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:sheetFormatPr defaultRowHeight="15"/>
-  <x:cols>
-    <x:col min="1" max="1" width="11.880000114440918" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="11.880000114440918" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="12.380000114440918" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="11.880000114440918" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="11.880000114440918" hidden="0" customWidth="1"/>
-  </x:cols>
-  <x:sheetData>
-    <x:row r="1">
-      <x:c r="A1" s="5" t="str">
-        <x:v>Fecha</x:v>
-      </x:c>
-      <x:c r="B1" s="5" t="str">
-        <x:v>Anio</x:v>
-      </x:c>
-      <x:c r="C1" s="5" t="str">
-        <x:v>MesNumero</x:v>
-      </x:c>
-      <x:c r="D1" s="5" t="str">
-        <x:v>Mes</x:v>
-      </x:c>
-      <x:c r="E1" s="5" t="str">
-        <x:v>TipoDia</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="2">
-      <x:c r="A2" s="6" t="str">
-        <x:v>2025-01-01</x:v>
-      </x:c>
-      <x:c r="B2" s="6" t="n">
-        <x:v>2025</x:v>
-      </x:c>
-      <x:c r="C2" s="6" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="D2" s="6" t="str">
-        <x:v>Ene</x:v>
-      </x:c>
-      <x:c r="E2" s="6" t="str">
-        <x:v>Laboral</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="3">
-      <x:c r="A3" s="6" t="str">
-        <x:v>2025-01-02</x:v>
-      </x:c>
-      <x:c r="B3" s="6" t="n">
-        <x:v>2025</x:v>
-      </x:c>
-      <x:c r="C3" s="6" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="D3" s="6" t="str">
-        <x:v>Ene</x:v>
-      </x:c>
-      <x:c r="E3" s="6" t="str">
-        <x:v>Laboral</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="4">
-      <x:c r="A4" s="6" t="str">
-        <x:v>2025-01-03</x:v>
-      </x:c>
-      <x:c r="B4" s="6" t="n">
-        <x:v>2025</x:v>
-      </x:c>
-      <x:c r="C4" s="6" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="D4" s="6" t="str">
-        <x:v>Ene</x:v>
-      </x:c>
-      <x:c r="E4" s="6" t="str">
-        <x:v>Laboral</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5">
-      <x:c r="A5" s="6" t="str">
-        <x:v>2025-01-04</x:v>
-      </x:c>
-      <x:c r="B5" s="6" t="n">
-        <x:v>2025</x:v>
-      </x:c>
-      <x:c r="C5" s="6" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="D5" s="6" t="str">
-        <x:v>Ene</x:v>
-      </x:c>
-      <x:c r="E5" s="6" t="str">
-        <x:v>Fin de semana</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6">
-      <x:c r="A6" s="6" t="str">
-        <x:v>2025-01-05</x:v>
-      </x:c>
-      <x:c r="B6" s="6" t="n">
-        <x:v>2025</x:v>
-      </x:c>
-      <x:c r="C6" s="6" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="D6" s="6" t="str">
-        <x:v>Ene</x:v>
-      </x:c>
-      <x:c r="E6" s="6" t="str">
-        <x:v>Fin de semana</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7">
-      <x:c r="A7" s="6" t="str">
-        <x:v>2025-01-06</x:v>
-      </x:c>
-      <x:c r="B7" s="6" t="n">
-        <x:v>2025</x:v>
-      </x:c>
-      <x:c r="C7" s="6" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="D7" s="6" t="str">
-        <x:v>Ene</x:v>
-      </x:c>
-      <x:c r="E7" s="6" t="str">
-        <x:v>Laboral</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8">
-      <x:c r="A8" s="6" t="str">
-        <x:v>2025-01-07</x:v>
-      </x:c>
-      <x:c r="B8" s="6" t="n">
-        <x:v>2025</x:v>
-      </x:c>
-      <x:c r="C8" s="6" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="D8" s="6" t="str">
-        <x:v>Ene</x:v>
-      </x:c>
-      <x:c r="E8" s="6" t="str">
-        <x:v>Laboral</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9">
-      <x:c r="A9" s="6" t="str">
-        <x:v>2025-01-08</x:v>
-      </x:c>
-      <x:c r="B9" s="6" t="n">
-        <x:v>2025</x:v>
-      </x:c>
-      <x:c r="C9" s="6" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="D9" s="6" t="str">
-        <x:v>Ene</x:v>
-      </x:c>
-      <x:c r="E9" s="6" t="str">
-        <x:v>Laboral</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="10">
-      <x:c r="A10" s="6" t="str">
-        <x:v>2025-01-09</x:v>
-      </x:c>
-      <x:c r="B10" s="6" t="n">
-        <x:v>2025</x:v>
-      </x:c>
-      <x:c r="C10" s="6" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="D10" s="6" t="str">
-        <x:v>Ene</x:v>
-      </x:c>
-      <x:c r="E10" s="6" t="str">
-        <x:v>Laboral</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="11">
-      <x:c r="A11" s="6" t="str">
-        <x:v>2025-01-10</x:v>
-      </x:c>
-      <x:c r="B11" s="6" t="n">
-        <x:v>2025</x:v>
-      </x:c>
-      <x:c r="C11" s="6" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="D11" s="6" t="str">
-        <x:v>Ene</x:v>
-      </x:c>
-      <x:c r="E11" s="6" t="str">
-        <x:v>Laboral</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="12">
-      <x:c r="A12" s="6" t="str">
-        <x:v>2025-01-11</x:v>
-      </x:c>
-      <x:c r="B12" s="6" t="n">
-        <x:v>2025</x:v>
-      </x:c>
-      <x:c r="C12" s="6" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="D12" s="6" t="str">
-        <x:v>Ene</x:v>
-      </x:c>
-      <x:c r="E12" s="6" t="str">
-        <x:v>Fin de semana</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="13">
-      <x:c r="A13" s="6" t="str">
-        <x:v>2025-01-12</x:v>
-      </x:c>
-      <x:c r="B13" s="6" t="n">
-        <x:v>2025</x:v>
-      </x:c>
-      <x:c r="C13" s="6" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="D13" s="6" t="str">
-        <x:v>Ene</x:v>
-      </x:c>
-      <x:c r="E13" s="6" t="str">
-        <x:v>Fin de semana</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="14">
-      <x:c r="A14" s="6" t="str">
-        <x:v>2025-01-13</x:v>
-      </x:c>
-      <x:c r="B14" s="6" t="n">
-        <x:v>2025</x:v>
-      </x:c>
-      <x:c r="C14" s="6" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="D14" s="6" t="str">
-        <x:v>Ene</x:v>
-      </x:c>
-      <x:c r="E14" s="6" t="str">
-        <x:v>Laboral</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="15">
-      <x:c r="A15" s="6" t="str">
-        <x:v>2025-01-14</x:v>
-      </x:c>
-      <x:c r="B15" s="6" t="n">
-        <x:v>2025</x:v>
-      </x:c>
-      <x:c r="C15" s="6" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="D15" s="6" t="str">
-        <x:v>Ene</x:v>
-      </x:c>
-      <x:c r="E15" s="6" t="str">
-        <x:v>Laboral</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="16">
-      <x:c r="A16" s="6" t="str">
-        <x:v>2025-01-15</x:v>
-      </x:c>
-      <x:c r="B16" s="6" t="n">
-        <x:v>2025</x:v>
-      </x:c>
-      <x:c r="C16" s="6" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="D16" s="6" t="str">
-        <x:v>Ene</x:v>
-      </x:c>
-      <x:c r="E16" s="6" t="str">
-        <x:v>Laboral</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="17">
-      <x:c r="A17" s="6" t="str">
-        <x:v>2025-01-16</x:v>
-      </x:c>
-      <x:c r="B17" s="6" t="n">
-        <x:v>2025</x:v>
-      </x:c>
-      <x:c r="C17" s="6" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="D17" s="6" t="str">
-        <x:v>Ene</x:v>
-      </x:c>
-      <x:c r="E17" s="6" t="str">
-        <x:v>Laboral</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="18">
-      <x:c r="A18" s="6" t="str">
-        <x:v>2025-01-17</x:v>
-      </x:c>
-      <x:c r="B18" s="6" t="n">
-        <x:v>2025</x:v>
-      </x:c>
-      <x:c r="C18" s="6" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="D18" s="6" t="str">
-        <x:v>Ene</x:v>
-      </x:c>
-      <x:c r="E18" s="6" t="str">
-        <x:v>Laboral</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="19">
-      <x:c r="A19" s="6" t="str">
-        <x:v>2025-01-18</x:v>
-      </x:c>
-      <x:c r="B19" s="6" t="n">
-        <x:v>2025</x:v>
-      </x:c>
-      <x:c r="C19" s="6" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="D19" s="6" t="str">
-        <x:v>Ene</x:v>
-      </x:c>
-      <x:c r="E19" s="6" t="str">
-        <x:v>Fin de semana</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="20">
-      <x:c r="A20" s="6" t="str">
-        <x:v>2025-01-19</x:v>
-      </x:c>
-      <x:c r="B20" s="6" t="n">
-        <x:v>2025</x:v>
-      </x:c>
-      <x:c r="C20" s="6" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="D20" s="6" t="str">
-        <x:v>Ene</x:v>
-      </x:c>
-      <x:c r="E20" s="6" t="str">
-        <x:v>Fin de semana</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="21">
-      <x:c r="A21" s="6" t="str">
-        <x:v>2025-01-20</x:v>
-      </x:c>
-      <x:c r="B21" s="6" t="n">
-        <x:v>2025</x:v>
-      </x:c>
-      <x:c r="C21" s="6" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="D21" s="6" t="str">
-        <x:v>Ene</x:v>
-      </x:c>
-      <x:c r="E21" s="6" t="str">
-        <x:v>Laboral</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="22">
-      <x:c r="A22" s="6" t="str">
-        <x:v>2025-01-21</x:v>
-      </x:c>
-      <x:c r="B22" s="6" t="n">
-        <x:v>2025</x:v>
-      </x:c>
-      <x:c r="C22" s="6" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="D22" s="6" t="str">
-        <x:v>Ene</x:v>
-      </x:c>
-      <x:c r="E22" s="6" t="str">
-        <x:v>Laboral</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="23">
-      <x:c r="A23" s="6" t="str">
-        <x:v>2025-01-22</x:v>
-      </x:c>
-      <x:c r="B23" s="6" t="n">
-        <x:v>2025</x:v>
-      </x:c>
-      <x:c r="C23" s="6" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="D23" s="6" t="str">
-        <x:v>Ene</x:v>
-      </x:c>
-      <x:c r="E23" s="6" t="str">
-        <x:v>Laboral</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="24">
-      <x:c r="A24" s="6" t="str">
-        <x:v>2025-01-23</x:v>
-      </x:c>
-      <x:c r="B24" s="6" t="n">
-        <x:v>2025</x:v>
-      </x:c>
-      <x:c r="C24" s="6" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="D24" s="6" t="str">
-        <x:v>Ene</x:v>
-      </x:c>
-      <x:c r="E24" s="6" t="str">
-        <x:v>Laboral</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="25">
-      <x:c r="A25" s="6" t="str">
-        <x:v>2025-01-24</x:v>
-      </x:c>
-      <x:c r="B25" s="6" t="n">
-        <x:v>2025</x:v>
-      </x:c>
-      <x:c r="C25" s="6" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="D25" s="6" t="str">
-        <x:v>Ene</x:v>
-      </x:c>
-      <x:c r="E25" s="6" t="str">
-        <x:v>Laboral</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="26">
-      <x:c r="A26" s="6" t="str">
-        <x:v>2025-01-25</x:v>
-      </x:c>
-      <x:c r="B26" s="6" t="n">
-        <x:v>2025</x:v>
-      </x:c>
-      <x:c r="C26" s="6" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="D26" s="6" t="str">
-        <x:v>Ene</x:v>
-      </x:c>
-      <x:c r="E26" s="6" t="str">
-        <x:v>Fin de semana</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="27">
-      <x:c r="A27" s="6" t="str">
-        <x:v>2025-01-26</x:v>
-      </x:c>
-      <x:c r="B27" s="6" t="n">
-        <x:v>2025</x:v>
-      </x:c>
-      <x:c r="C27" s="6" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="D27" s="6" t="str">
-        <x:v>Ene</x:v>
-      </x:c>
-      <x:c r="E27" s="6" t="str">
-        <x:v>Fin de semana</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="28">
-      <x:c r="A28" s="6" t="str">
-        <x:v>2025-01-27</x:v>
-      </x:c>
-      <x:c r="B28" s="6" t="n">
-        <x:v>2025</x:v>
-      </x:c>
-      <x:c r="C28" s="6" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="D28" s="6" t="str">
-        <x:v>Ene</x:v>
-      </x:c>
-      <x:c r="E28" s="6" t="str">
-        <x:v>Laboral</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="29">
-      <x:c r="A29" s="6" t="str">
-        <x:v>2025-01-28</x:v>
-      </x:c>
-      <x:c r="B29" s="6" t="n">
-        <x:v>2025</x:v>
-      </x:c>
-      <x:c r="C29" s="6" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="D29" s="6" t="str">
-        <x:v>Ene</x:v>
-      </x:c>
-      <x:c r="E29" s="6" t="str">
-        <x:v>Laboral</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="30">
-      <x:c r="A30" s="6" t="str">
-        <x:v>2025-01-29</x:v>
-      </x:c>
-      <x:c r="B30" s="6" t="n">
-        <x:v>2025</x:v>
-      </x:c>
-      <x:c r="C30" s="6" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="D30" s="6" t="str">
-        <x:v>Ene</x:v>
-      </x:c>
-      <x:c r="E30" s="6" t="str">
-        <x:v>Laboral</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="31">
-      <x:c r="A31" s="6" t="str">
-        <x:v>2025-01-30</x:v>
-      </x:c>
-      <x:c r="B31" s="6" t="n">
-        <x:v>2025</x:v>
-      </x:c>
-      <x:c r="C31" s="6" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="D31" s="6" t="str">
-        <x:v>Ene</x:v>
-      </x:c>
-      <x:c r="E31" s="6" t="str">
-        <x:v>Laboral</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="32">
-      <x:c r="A32" s="6" t="str">
-        <x:v>2025-01-31</x:v>
-      </x:c>
-      <x:c r="B32" s="6" t="n">
-        <x:v>2025</x:v>
-      </x:c>
-      <x:c r="C32" s="6" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="D32" s="6" t="str">
-        <x:v>Ene</x:v>
-      </x:c>
-      <x:c r="E32" s="6" t="str">
-        <x:v>Laboral</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="33">
-      <x:c r="A33" s="6" t="str">
-        <x:v>2025-02-01</x:v>
-      </x:c>
-      <x:c r="B33" s="6" t="n">
-        <x:v>2025</x:v>
-      </x:c>
-      <x:c r="C33" s="6" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="D33" s="6" t="str">
-        <x:v>Feb</x:v>
-      </x:c>
-      <x:c r="E33" s="6" t="str">
-        <x:v>Fin de semana</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="34">
-      <x:c r="A34" s="6" t="str">
-        <x:v>2025-02-02</x:v>
-      </x:c>
-      <x:c r="B34" s="6" t="n">
-        <x:v>2025</x:v>
-      </x:c>
-      <x:c r="C34" s="6" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="D34" s="6" t="str">
-        <x:v>Feb</x:v>
-      </x:c>
-      <x:c r="E34" s="6" t="str">
-        <x:v>Fin de semana</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="35">
-      <x:c r="A35" s="6" t="str">
-        <x:v>2025-02-03</x:v>
-      </x:c>
-      <x:c r="B35" s="6" t="n">
-        <x:v>2025</x:v>
-      </x:c>
-      <x:c r="C35" s="6" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="D35" s="6" t="str">
-        <x:v>Feb</x:v>
-      </x:c>
-      <x:c r="E35" s="6" t="str">
-        <x:v>Laboral</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="36">
-      <x:c r="A36" s="6" t="str">
-        <x:v>2025-02-04</x:v>
-      </x:c>
-      <x:c r="B36" s="6" t="n">
-        <x:v>2025</x:v>
-      </x:c>
-      <x:c r="C36" s="6" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="D36" s="6" t="str">
-        <x:v>Feb</x:v>
-      </x:c>
-      <x:c r="E36" s="6" t="str">
-        <x:v>Laboral</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="37">
-      <x:c r="A37" s="6" t="str">
-        <x:v>2025-02-05</x:v>
-      </x:c>
-      <x:c r="B37" s="6" t="n">
-        <x:v>2025</x:v>
-      </x:c>
-      <x:c r="C37" s="6" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="D37" s="6" t="str">
-        <x:v>Feb</x:v>
-      </x:c>
-      <x:c r="E37" s="6" t="str">
-        <x:v>Laboral</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="38">
-      <x:c r="A38" s="6" t="str">
-        <x:v>2025-02-06</x:v>
-      </x:c>
-      <x:c r="B38" s="6" t="n">
-        <x:v>2025</x:v>
-      </x:c>
-      <x:c r="C38" s="6" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="D38" s="6" t="str">
-        <x:v>Feb</x:v>
-      </x:c>
-      <x:c r="E38" s="6" t="str">
-        <x:v>Laboral</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="39">
-      <x:c r="A39" s="6" t="str">
-        <x:v>2025-02-07</x:v>
-      </x:c>
-      <x:c r="B39" s="6" t="n">
-        <x:v>2025</x:v>
-      </x:c>
-      <x:c r="C39" s="6" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="D39" s="6" t="str">
-        <x:v>Feb</x:v>
-      </x:c>
-      <x:c r="E39" s="6" t="str">
-        <x:v>Laboral</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="40">
-      <x:c r="A40" s="6" t="str">
-        <x:v>2025-02-08</x:v>
-      </x:c>
-      <x:c r="B40" s="6" t="n">
-        <x:v>2025</x:v>
-      </x:c>
-      <x:c r="C40" s="6" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="D40" s="6" t="str">
-        <x:v>Feb</x:v>
-      </x:c>
-      <x:c r="E40" s="6" t="str">
-        <x:v>Fin de semana</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="41">
-      <x:c r="A41" s="6" t="str">
-        <x:v>2025-02-09</x:v>
-      </x:c>
-      <x:c r="B41" s="6" t="n">
-        <x:v>2025</x:v>
-      </x:c>
-      <x:c r="C41" s="6" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="D41" s="6" t="str">
-        <x:v>Feb</x:v>
-      </x:c>
-      <x:c r="E41" s="6" t="str">
-        <x:v>Fin de semana</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="42">
-      <x:c r="A42" s="6" t="str">
-        <x:v>2025-02-10</x:v>
-      </x:c>
-      <x:c r="B42" s="6" t="n">
-        <x:v>2025</x:v>
-      </x:c>
-      <x:c r="C42" s="6" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="D42" s="6" t="str">
-        <x:v>Feb</x:v>
-      </x:c>
-      <x:c r="E42" s="6" t="str">
-        <x:v>Laboral</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="43">
-      <x:c r="A43" s="6" t="str">
-        <x:v>2025-02-11</x:v>
-      </x:c>
-      <x:c r="B43" s="6" t="n">
-        <x:v>2025</x:v>
-      </x:c>
-      <x:c r="C43" s="6" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="D43" s="6" t="str">
-        <x:v>Feb</x:v>
-      </x:c>
-      <x:c r="E43" s="6" t="str">
-        <x:v>Laboral</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="44">
-      <x:c r="A44" s="6" t="str">
-        <x:v>2025-02-12</x:v>
-      </x:c>
-      <x:c r="B44" s="6" t="n">
-        <x:v>2025</x:v>
-      </x:c>
-      <x:c r="C44" s="6" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="D44" s="6" t="str">
-        <x:v>Feb</x:v>
-      </x:c>
-      <x:c r="E44" s="6" t="str">
-        <x:v>Laboral</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="45">
-      <x:c r="A45" s="6" t="str">
-        <x:v>2025-02-13</x:v>
-      </x:c>
-      <x:c r="B45" s="6" t="n">
-        <x:v>2025</x:v>
-      </x:c>
-      <x:c r="C45" s="6" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="D45" s="6" t="str">
-        <x:v>Feb</x:v>
-      </x:c>
-      <x:c r="E45" s="6" t="str">
-        <x:v>Laboral</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="46">
-      <x:c r="A46" s="6" t="str">
-        <x:v>2025-02-14</x:v>
-      </x:c>
-      <x:c r="B46" s="6" t="n">
-        <x:v>2025</x:v>
-      </x:c>
-      <x:c r="C46" s="6" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="D46" s="6" t="str">
-        <x:v>Feb</x:v>
-      </x:c>
-      <x:c r="E46" s="6" t="str">
-        <x:v>Laboral</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="47">
-      <x:c r="A47" s="6" t="str">
-        <x:v>2025-02-15</x:v>
-      </x:c>
-      <x:c r="B47" s="6" t="n">
-        <x:v>2025</x:v>
-      </x:c>
-      <x:c r="C47" s="6" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="D47" s="6" t="str">
-        <x:v>Feb</x:v>
-      </x:c>
-      <x:c r="E47" s="6" t="str">
-        <x:v>Fin de semana</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="48">
-      <x:c r="A48" s="6" t="str">
-        <x:v>2025-02-16</x:v>
-      </x:c>
-      <x:c r="B48" s="6" t="n">
-        <x:v>2025</x:v>
-      </x:c>
-      <x:c r="C48" s="6" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="D48" s="6" t="str">
-        <x:v>Feb</x:v>
-      </x:c>
-      <x:c r="E48" s="6" t="str">
-        <x:v>Fin de semana</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="49">
-      <x:c r="A49" s="6" t="str">
-        <x:v>2025-02-17</x:v>
-      </x:c>
-      <x:c r="B49" s="6" t="n">
-        <x:v>2025</x:v>
-      </x:c>
-      <x:c r="C49" s="6" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="D49" s="6" t="str">
-        <x:v>Feb</x:v>
-      </x:c>
-      <x:c r="E49" s="6" t="str">
-        <x:v>Laboral</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="50">
-      <x:c r="A50" s="6" t="str">
-        <x:v>2025-02-18</x:v>
-      </x:c>
-      <x:c r="B50" s="6" t="n">
-        <x:v>2025</x:v>
-      </x:c>
-      <x:c r="C50" s="6" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="D50" s="6" t="str">
-        <x:v>Feb</x:v>
-      </x:c>
-      <x:c r="E50" s="6" t="str">
-        <x:v>Laboral</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="51">
-      <x:c r="A51" s="6" t="str">
-        <x:v>2025-02-19</x:v>
-      </x:c>
-      <x:c r="B51" s="6" t="n">
-        <x:v>2025</x:v>
-      </x:c>
-      <x:c r="C51" s="6" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="D51" s="6" t="str">
-        <x:v>Feb</x:v>
-      </x:c>
-      <x:c r="E51" s="6" t="str">
-        <x:v>Laboral</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="52">
-      <x:c r="A52" s="6" t="str">
-        <x:v>2025-02-20</x:v>
-      </x:c>
-      <x:c r="B52" s="6" t="n">
-        <x:v>2025</x:v>
-      </x:c>
-      <x:c r="C52" s="6" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="D52" s="6" t="str">
-        <x:v>Feb</x:v>
-      </x:c>
-      <x:c r="E52" s="6" t="str">
-        <x:v>Laboral</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="53">
-      <x:c r="A53" s="6" t="str">
-        <x:v>2025-02-21</x:v>
-      </x:c>
-      <x:c r="B53" s="6" t="n">
-        <x:v>2025</x:v>
-      </x:c>
-      <x:c r="C53" s="6" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="D53" s="6" t="str">
-        <x:v>Feb</x:v>
-      </x:c>
-      <x:c r="E53" s="6" t="str">
-        <x:v>Laboral</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="54">
-      <x:c r="A54" s="6" t="str">
-        <x:v>2025-02-22</x:v>
-      </x:c>
-      <x:c r="B54" s="6" t="n">
-        <x:v>2025</x:v>
-      </x:c>
-      <x:c r="C54" s="6" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="D54" s="6" t="str">
-        <x:v>Feb</x:v>
-      </x:c>
-      <x:c r="E54" s="6" t="str">
-        <x:v>Fin de semana</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="55">
-      <x:c r="A55" s="6" t="str">
-        <x:v>2025-02-23</x:v>
-      </x:c>
-      <x:c r="B55" s="6" t="n">
-        <x:v>2025</x:v>
-      </x:c>
-      <x:c r="C55" s="6" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="D55" s="6" t="str">
-        <x:v>Feb</x:v>
-      </x:c>
-      <x:c r="E55" s="6" t="str">
-        <x:v>Fin de semana</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="56">
-      <x:c r="A56" s="6" t="str">
-        <x:v>2025-02-24</x:v>
-      </x:c>
-      <x:c r="B56" s="6" t="n">
-        <x:v>2025</x:v>
-      </x:c>
-      <x:c r="C56" s="6" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="D56" s="6" t="str">
-        <x:v>Feb</x:v>
-      </x:c>
-      <x:c r="E56" s="6" t="str">
-        <x:v>Laboral</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="57">
-      <x:c r="A57" s="6" t="str">
-        <x:v>2025-02-25</x:v>
-      </x:c>
-      <x:c r="B57" s="6" t="n">
-        <x:v>2025</x:v>
-      </x:c>
-      <x:c r="C57" s="6" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="D57" s="6" t="str">
-        <x:v>Feb</x:v>
-      </x:c>
-      <x:c r="E57" s="6" t="str">
-        <x:v>Laboral</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="58">
-      <x:c r="A58" s="6" t="str">
-        <x:v>2025-02-26</x:v>
-      </x:c>
-      <x:c r="B58" s="6" t="n">
-        <x:v>2025</x:v>
-      </x:c>
-      <x:c r="C58" s="6" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="D58" s="6" t="str">
-        <x:v>Feb</x:v>
-      </x:c>
-      <x:c r="E58" s="6" t="str">
-        <x:v>Laboral</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="59">
-      <x:c r="A59" s="6" t="str">
-        <x:v>2025-02-27</x:v>
-      </x:c>
-      <x:c r="B59" s="6" t="n">
-        <x:v>2025</x:v>
-      </x:c>
-      <x:c r="C59" s="6" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="D59" s="6" t="str">
-        <x:v>Feb</x:v>
-      </x:c>
-      <x:c r="E59" s="6" t="str">
-        <x:v>Laboral</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="60">
-      <x:c r="A60" s="6" t="str">
-        <x:v>2025-02-28</x:v>
-      </x:c>
-      <x:c r="B60" s="6" t="n">
-        <x:v>2025</x:v>
-      </x:c>
-      <x:c r="C60" s="6" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="D60" s="6" t="str">
-        <x:v>Feb</x:v>
-      </x:c>
-      <x:c r="E60" s="6" t="str">
-        <x:v>Laboral</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="61">
-      <x:c r="A61" s="6" t="str">
-        <x:v>2025-03-01</x:v>
-      </x:c>
-      <x:c r="B61" s="6" t="n">
-        <x:v>2025</x:v>
-      </x:c>
-      <x:c r="C61" s="6" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="D61" s="6" t="str">
-        <x:v>Mar</x:v>
-      </x:c>
-      <x:c r="E61" s="6" t="str">
-        <x:v>Fin de semana</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="62">
-      <x:c r="A62" s="6" t="str">
-        <x:v>2025-03-02</x:v>
-      </x:c>
-      <x:c r="B62" s="6" t="n">
-        <x:v>2025</x:v>
-      </x:c>
-      <x:c r="C62" s="6" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="D62" s="6" t="str">
-        <x:v>Mar</x:v>
-      </x:c>
-      <x:c r="E62" s="6" t="str">
-        <x:v>Fin de semana</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="63">
-      <x:c r="A63" s="6" t="str">
-        <x:v>2025-03-03</x:v>
-      </x:c>
-      <x:c r="B63" s="6" t="n">
-        <x:v>2025</x:v>
-      </x:c>
-      <x:c r="C63" s="6" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="D63" s="6" t="str">
-        <x:v>Mar</x:v>
-      </x:c>
-      <x:c r="E63" s="6" t="str">
-        <x:v>Laboral</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="64">
-      <x:c r="A64" s="6" t="str">
-        <x:v>2025-03-04</x:v>
-      </x:c>
-      <x:c r="B64" s="6" t="n">
-        <x:v>2025</x:v>
-      </x:c>
-      <x:c r="C64" s="6" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="D64" s="6" t="str">
-        <x:v>Mar</x:v>
-      </x:c>
-      <x:c r="E64" s="6" t="str">
-        <x:v>Laboral</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="65">
-      <x:c r="A65" s="6" t="str">
-        <x:v>2025-03-05</x:v>
-      </x:c>
-      <x:c r="B65" s="6" t="n">
-        <x:v>2025</x:v>
-      </x:c>
-      <x:c r="C65" s="6" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="D65" s="6" t="str">
-        <x:v>Mar</x:v>
-      </x:c>
-      <x:c r="E65" s="6" t="str">
-        <x:v>Laboral</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="66">
-      <x:c r="A66" s="6" t="str">
-        <x:v>2025-03-06</x:v>
-      </x:c>
-      <x:c r="B66" s="6" t="n">
-        <x:v>2025</x:v>
-      </x:c>
-      <x:c r="C66" s="6" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="D66" s="6" t="str">
-        <x:v>Mar</x:v>
-      </x:c>
-      <x:c r="E66" s="6" t="str">
-        <x:v>Laboral</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="67">
-      <x:c r="A67" s="6" t="str">
-        <x:v>2025-03-07</x:v>
-      </x:c>
-      <x:c r="B67" s="6" t="n">
-        <x:v>2025</x:v>
-      </x:c>
-      <x:c r="C67" s="6" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="D67" s="6" t="str">
-        <x:v>Mar</x:v>
-      </x:c>
-      <x:c r="E67" s="6" t="str">
-        <x:v>Laboral</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="68">
-      <x:c r="A68" s="6" t="str">
-        <x:v>2025-03-08</x:v>
-      </x:c>
-      <x:c r="B68" s="6" t="n">
-        <x:v>2025</x:v>
-      </x:c>
-      <x:c r="C68" s="6" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="D68" s="6" t="str">
-        <x:v>Mar</x:v>
-      </x:c>
-      <x:c r="E68" s="6" t="str">
-        <x:v>Fin de semana</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="69">
-      <x:c r="A69" s="6" t="str">
-        <x:v>2025-03-09</x:v>
-      </x:c>
-      <x:c r="B69" s="6" t="n">
-        <x:v>2025</x:v>
-      </x:c>
-      <x:c r="C69" s="6" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="D69" s="6" t="str">
-        <x:v>Mar</x:v>
-      </x:c>
-      <x:c r="E69" s="6" t="str">
-        <x:v>Fin de semana</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="70">
-      <x:c r="A70" s="6" t="str">
-        <x:v>2025-03-10</x:v>
-      </x:c>
-      <x:c r="B70" s="6" t="n">
-        <x:v>2025</x:v>
-      </x:c>
-      <x:c r="C70" s="6" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="D70" s="6" t="str">
-        <x:v>Mar</x:v>
-      </x:c>
-      <x:c r="E70" s="6" t="str">
-        <x:v>Laboral</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="71">
-      <x:c r="A71" s="6" t="str">
-        <x:v>2025-03-11</x:v>
-      </x:c>
-      <x:c r="B71" s="6" t="n">
-        <x:v>2025</x:v>
-      </x:c>
-      <x:c r="C71" s="6" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="D71" s="6" t="str">
-        <x:v>Mar</x:v>
-      </x:c>
-      <x:c r="E71" s="6" t="str">
-        <x:v>Laboral</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="72">
-      <x:c r="A72" s="6" t="str">
-        <x:v>2025-03-12</x:v>
-      </x:c>
-      <x:c r="B72" s="6" t="n">
-        <x:v>2025</x:v>
-      </x:c>
-      <x:c r="C72" s="6" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="D72" s="6" t="str">
-        <x:v>Mar</x:v>
-      </x:c>
-      <x:c r="E72" s="6" t="str">
-        <x:v>Laboral</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="73">
-      <x:c r="A73" s="6" t="str">
-        <x:v>2025-03-13</x:v>
-      </x:c>
-      <x:c r="B73" s="6" t="n">
-        <x:v>2025</x:v>
-      </x:c>
-      <x:c r="C73" s="6" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="D73" s="6" t="str">
-        <x:v>Mar</x:v>
-      </x:c>
-      <x:c r="E73" s="6" t="str">
-        <x:v>Laboral</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="74">
-      <x:c r="A74" s="6" t="str">
-        <x:v>2025-03-14</x:v>
-      </x:c>
-      <x:c r="B74" s="6" t="n">
-        <x:v>2025</x:v>
-      </x:c>
-      <x:c r="C74" s="6" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="D74" s="6" t="str">
-        <x:v>Mar</x:v>
-      </x:c>
-      <x:c r="E74" s="6" t="str">
-        <x:v>Laboral</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="75">
-      <x:c r="A75" s="6" t="str">
-        <x:v>2025-03-15</x:v>
-      </x:c>
-      <x:c r="B75" s="6" t="n">
-        <x:v>2025</x:v>
-      </x:c>
-      <x:c r="C75" s="6" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="D75" s="6" t="str">
-        <x:v>Mar</x:v>
-      </x:c>
-      <x:c r="E75" s="6" t="str">
-        <x:v>Fin de semana</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="76">
-      <x:c r="A76" s="6" t="str">
-        <x:v>2025-03-16</x:v>
-      </x:c>
-      <x:c r="B76" s="6" t="n">
-        <x:v>2025</x:v>
-      </x:c>
-      <x:c r="C76" s="6" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="D76" s="6" t="str">
-        <x:v>Mar</x:v>
-      </x:c>
-      <x:c r="E76" s="6" t="str">
-        <x:v>Fin de semana</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="77">
-      <x:c r="A77" s="6" t="str">
-        <x:v>2025-03-17</x:v>
-      </x:c>
-      <x:c r="B77" s="6" t="n">
-        <x:v>2025</x:v>
-      </x:c>
-      <x:c r="C77" s="6" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="D77" s="6" t="str">
-        <x:v>Mar</x:v>
-      </x:c>
-      <x:c r="E77" s="6" t="str">
-        <x:v>Laboral</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="78">
-      <x:c r="A78" s="6" t="str">
-        <x:v>2025-03-18</x:v>
-      </x:c>
-      <x:c r="B78" s="6" t="n">
-        <x:v>2025</x:v>
-      </x:c>
-      <x:c r="C78" s="6" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="D78" s="6" t="str">
-        <x:v>Mar</x:v>
-      </x:c>
-      <x:c r="E78" s="6" t="str">
-        <x:v>Laboral</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="79">
-      <x:c r="A79" s="6" t="str">
-        <x:v>2025-03-19</x:v>
-      </x:c>
-      <x:c r="B79" s="6" t="n">
-        <x:v>2025</x:v>
-      </x:c>
-      <x:c r="C79" s="6" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="D79" s="6" t="str">
-        <x:v>Mar</x:v>
-      </x:c>
-      <x:c r="E79" s="6" t="str">
-        <x:v>Laboral</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="80">
-      <x:c r="A80" s="6" t="str">
-        <x:v>2025-03-20</x:v>
-      </x:c>
-      <x:c r="B80" s="6" t="n">
-        <x:v>2025</x:v>
-      </x:c>
-      <x:c r="C80" s="6" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="D80" s="6" t="str">
-        <x:v>Mar</x:v>
-      </x:c>
-      <x:c r="E80" s="6" t="str">
-        <x:v>Laboral</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="81">
-      <x:c r="A81" s="6" t="str">
-        <x:v>2025-03-21</x:v>
-      </x:c>
-      <x:c r="B81" s="6" t="n">
-        <x:v>2025</x:v>
-      </x:c>
-      <x:c r="C81" s="6" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="D81" s="6" t="str">
-        <x:v>Mar</x:v>
-      </x:c>
-      <x:c r="E81" s="6" t="str">
-        <x:v>Laboral</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="82">
-      <x:c r="A82" s="6" t="str">
-        <x:v>2025-03-22</x:v>
-      </x:c>
-      <x:c r="B82" s="6" t="n">
-        <x:v>2025</x:v>
-      </x:c>
-      <x:c r="C82" s="6" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="D82" s="6" t="str">
-        <x:v>Mar</x:v>
-      </x:c>
-      <x:c r="E82" s="6" t="str">
-        <x:v>Fin de semana</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="83">
-      <x:c r="A83" s="6" t="str">
-        <x:v>2025-03-23</x:v>
-      </x:c>
-      <x:c r="B83" s="6" t="n">
-        <x:v>2025</x:v>
-      </x:c>
-      <x:c r="C83" s="6" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="D83" s="6" t="str">
-        <x:v>Mar</x:v>
-      </x:c>
-      <x:c r="E83" s="6" t="str">
-        <x:v>Fin de semana</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="84">
-      <x:c r="A84" s="6" t="str">
-        <x:v>2025-03-24</x:v>
-      </x:c>
-      <x:c r="B84" s="6" t="n">
-        <x:v>2025</x:v>
-      </x:c>
-      <x:c r="C84" s="6" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="D84" s="6" t="str">
-        <x:v>Mar</x:v>
-      </x:c>
-      <x:c r="E84" s="6" t="str">
-        <x:v>Laboral</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="85">
-      <x:c r="A85" s="6" t="str">
-        <x:v>2025-03-25</x:v>
-      </x:c>
-      <x:c r="B85" s="6" t="n">
-        <x:v>2025</x:v>
-      </x:c>
-      <x:c r="C85" s="6" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="D85" s="6" t="str">
-        <x:v>Mar</x:v>
-      </x:c>
-      <x:c r="E85" s="6" t="str">
-        <x:v>Laboral</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="86">
-      <x:c r="A86" s="6" t="str">
-        <x:v>2025-03-26</x:v>
-      </x:c>
-      <x:c r="B86" s="6" t="n">
-        <x:v>2025</x:v>
-      </x:c>
-      <x:c r="C86" s="6" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="D86" s="6" t="str">
-        <x:v>Mar</x:v>
-      </x:c>
-      <x:c r="E86" s="6" t="str">
-        <x:v>Laboral</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="87">
-      <x:c r="A87" s="6" t="str">
-        <x:v>2025-03-27</x:v>
-      </x:c>
-      <x:c r="B87" s="6" t="n">
-        <x:v>2025</x:v>
-      </x:c>
-      <x:c r="C87" s="6" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="D87" s="6" t="str">
-        <x:v>Mar</x:v>
-      </x:c>
-      <x:c r="E87" s="6" t="str">
-        <x:v>Laboral</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="88">
-      <x:c r="A88" s="6" t="str">
-        <x:v>2025-03-28</x:v>
-      </x:c>
-      <x:c r="B88" s="6" t="n">
-        <x:v>2025</x:v>
-      </x:c>
-      <x:c r="C88" s="6" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="D88" s="6" t="str">
-        <x:v>Mar</x:v>
-      </x:c>
-      <x:c r="E88" s="6" t="str">
-        <x:v>Laboral</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="89">
-      <x:c r="A89" s="6" t="str">
-        <x:v>2025-03-29</x:v>
-      </x:c>
-      <x:c r="B89" s="6" t="n">
-        <x:v>2025</x:v>
-      </x:c>
-      <x:c r="C89" s="6" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="D89" s="6" t="str">
-        <x:v>Mar</x:v>
-      </x:c>
-      <x:c r="E89" s="6" t="str">
-        <x:v>Fin de semana</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="90">
-      <x:c r="A90" s="6" t="str">
-        <x:v>2025-03-30</x:v>
-      </x:c>
-      <x:c r="B90" s="6" t="n">
-        <x:v>2025</x:v>
-      </x:c>
-      <x:c r="C90" s="6" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="D90" s="6" t="str">
-        <x:v>Mar</x:v>
-      </x:c>
-      <x:c r="E90" s="6" t="str">
-        <x:v>Fin de semana</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="91">
-      <x:c r="A91" s="6" t="str">
-        <x:v>2025-03-31</x:v>
-      </x:c>
-      <x:c r="B91" s="6" t="n">
-        <x:v>2025</x:v>
-      </x:c>
-      <x:c r="C91" s="6" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="D91" s="6" t="str">
-        <x:v>Mar</x:v>
-      </x:c>
-      <x:c r="E91" s="6" t="str">
-        <x:v>Laboral</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="92">
-      <x:c r="A92" s="6" t="str">
-        <x:v>2025-04-01</x:v>
-      </x:c>
-      <x:c r="B92" s="6" t="n">
-        <x:v>2025</x:v>
-      </x:c>
-      <x:c r="C92" s="6" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="D92" s="6" t="str">
-        <x:v>Abr</x:v>
-      </x:c>
-      <x:c r="E92" s="6" t="str">
-        <x:v>Laboral</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="93">
-      <x:c r="A93" s="6" t="str">
-        <x:v>2025-04-02</x:v>
-      </x:c>
-      <x:c r="B93" s="6" t="n">
-        <x:v>2025</x:v>
-      </x:c>
-      <x:c r="C93" s="6" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="D93" s="6" t="str">
-        <x:v>Abr</x:v>
-      </x:c>
-      <x:c r="E93" s="6" t="str">
-        <x:v>Laboral</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="94">
-      <x:c r="A94" s="6" t="str">
-        <x:v>2025-04-03</x:v>
-      </x:c>
-      <x:c r="B94" s="6" t="n">
-        <x:v>2025</x:v>
-      </x:c>
-      <x:c r="C94" s="6" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="D94" s="6" t="str">
-        <x:v>Abr</x:v>
-      </x:c>
-      <x:c r="E94" s="6" t="str">
-        <x:v>Laboral</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="95">
-      <x:c r="A95" s="6" t="str">
-        <x:v>2025-04-04</x:v>
-      </x:c>
-      <x:c r="B95" s="6" t="n">
-        <x:v>2025</x:v>
-      </x:c>
-      <x:c r="C95" s="6" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="D95" s="6" t="str">
-        <x:v>Abr</x:v>
-      </x:c>
-      <x:c r="E95" s="6" t="str">
-        <x:v>Laboral</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="96">
-      <x:c r="A96" s="6" t="str">
-        <x:v>2025-04-05</x:v>
-      </x:c>
-      <x:c r="B96" s="6" t="n">
-        <x:v>2025</x:v>
-      </x:c>
-      <x:c r="C96" s="6" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="D96" s="6" t="str">
-        <x:v>Abr</x:v>
-      </x:c>
-      <x:c r="E96" s="6" t="str">
-        <x:v>Fin de semana</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="97">
-      <x:c r="A97" s="6" t="str">
-        <x:v>2025-04-06</x:v>
-      </x:c>
-      <x:c r="B97" s="6" t="n">
-        <x:v>2025</x:v>
-      </x:c>
-      <x:c r="C97" s="6" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="D97" s="6" t="str">
-        <x:v>Abr</x:v>
-      </x:c>
-      <x:c r="E97" s="6" t="str">
-        <x:v>Fin de semana</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="98">
-      <x:c r="A98" s="6" t="str">
-        <x:v>2025-04-07</x:v>
-      </x:c>
-      <x:c r="B98" s="6" t="n">
-        <x:v>2025</x:v>
-      </x:c>
-      <x:c r="C98" s="6" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="D98" s="6" t="str">
-        <x:v>Abr</x:v>
-      </x:c>
-      <x:c r="E98" s="6" t="str">
-        <x:v>Laboral</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="99">
-      <x:c r="A99" s="6" t="str">
-        <x:v>2025-04-08</x:v>
-      </x:c>
-      <x:c r="B99" s="6" t="n">
-        <x:v>2025</x:v>
-      </x:c>
-      <x:c r="C99" s="6" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="D99" s="6" t="str">
-        <x:v>Abr</x:v>
-      </x:c>
-      <x:c r="E99" s="6" t="str">
-        <x:v>Laboral</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="100">
-      <x:c r="A100" s="6" t="str">
-        <x:v>2025-04-09</x:v>
-      </x:c>
-      <x:c r="B100" s="6" t="n">
-        <x:v>2025</x:v>
-      </x:c>
-      <x:c r="C100" s="6" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="D100" s="6" t="str">
-        <x:v>Abr</x:v>
-      </x:c>
-      <x:c r="E100" s="6" t="str">
-        <x:v>Laboral</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="101">
-      <x:c r="A101" s="6" t="str">
-        <x:v>2025-04-10</x:v>
-      </x:c>
-      <x:c r="B101" s="6" t="n">
-        <x:v>2025</x:v>
-      </x:c>
-      <x:c r="C101" s="6" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="D101" s="6" t="str">
-        <x:v>Abr</x:v>
-      </x:c>
-      <x:c r="E101" s="6" t="str">
-        <x:v>Laboral</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="102">
-      <x:c r="A102" s="6" t="str">
-        <x:v>2025-04-11</x:v>
-      </x:c>
-      <x:c r="B102" s="6" t="n">
-        <x:v>2025</x:v>
-      </x:c>
-      <x:c r="C102" s="6" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="D102" s="6" t="str">
-        <x:v>Abr</x:v>
-      </x:c>
-      <x:c r="E102" s="6" t="str">
-        <x:v>Laboral</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="103">
-      <x:c r="A103" s="6" t="str">
-        <x:v>2025-04-12</x:v>
-      </x:c>
-      <x:c r="B103" s="6" t="n">
-        <x:v>2025</x:v>
-      </x:c>
-      <x:c r="C103" s="6" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="D103" s="6" t="str">
-        <x:v>Abr</x:v>
-      </x:c>
-      <x:c r="E103" s="6" t="str">
-        <x:v>Fin de semana</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="104">
-      <x:c r="A104" s="6" t="str">
-        <x:v>2025-04-13</x:v>
-      </x:c>
-      <x:c r="B104" s="6" t="n">
-        <x:v>2025</x:v>
-      </x:c>
-      <x:c r="C104" s="6" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="D104" s="6" t="str">
-        <x:v>Abr</x:v>
-      </x:c>
-      <x:c r="E104" s="6" t="str">
-        <x:v>Fin de semana</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="105">
-      <x:c r="A105" s="6" t="str">
-        <x:v>2025-04-14</x:v>
-      </x:c>
-      <x:c r="B105" s="6" t="n">
-        <x:v>2025</x:v>
-      </x:c>
-      <x:c r="C105" s="6" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="D105" s="6" t="str">
-        <x:v>Abr</x:v>
-      </x:c>
-      <x:c r="E105" s="6" t="str">
-        <x:v>Laboral</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="106">
-      <x:c r="A106" s="6" t="str">
-        <x:v>2025-04-15</x:v>
-      </x:c>
-      <x:c r="B106" s="6" t="n">
-        <x:v>2025</x:v>
-      </x:c>
-      <x:c r="C106" s="6" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="D106" s="6" t="str">
-        <x:v>Abr</x:v>
-      </x:c>
-      <x:c r="E106" s="6" t="str">
-        <x:v>Laboral</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="107">
-      <x:c r="A107" s="6" t="str">
-        <x:v>2025-04-16</x:v>
-      </x:c>
-      <x:c r="B107" s="6" t="n">
-        <x:v>2025</x:v>
-      </x:c>
-      <x:c r="C107" s="6" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="D107" s="6" t="str">
-        <x:v>Abr</x:v>
-      </x:c>
-      <x:c r="E107" s="6" t="str">
-        <x:v>Laboral</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="108">
-      <x:c r="A108" s="6" t="str">
-        <x:v>2025-04-17</x:v>
-      </x:c>
-      <x:c r="B108" s="6" t="n">
-        <x:v>2025</x:v>
-      </x:c>
-      <x:c r="C108" s="6" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="D108" s="6" t="str">
-        <x:v>Abr</x:v>
-      </x:c>
-      <x:c r="E108" s="6" t="str">
-        <x:v>Laboral</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="109">
-      <x:c r="A109" s="6" t="str">
-        <x:v>2025-04-18</x:v>
-      </x:c>
-      <x:c r="B109" s="6" t="n">
-        <x:v>2025</x:v>
-      </x:c>
-      <x:c r="C109" s="6" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="D109" s="6" t="str">
-        <x:v>Abr</x:v>
-      </x:c>
-      <x:c r="E109" s="6" t="str">
-        <x:v>Laboral</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="110">
-      <x:c r="A110" s="6" t="str">
-        <x:v>2025-04-19</x:v>
-      </x:c>
-      <x:c r="B110" s="6" t="n">
-        <x:v>2025</x:v>
-      </x:c>
-      <x:c r="C110" s="6" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="D110" s="6" t="str">
-        <x:v>Abr</x:v>
-      </x:c>
-      <x:c r="E110" s="6" t="str">
-        <x:v>Fin de semana</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="111">
-      <x:c r="A111" s="6" t="str">
-        <x:v>2025-04-20</x:v>
-      </x:c>
-      <x:c r="B111" s="6" t="n">
-        <x:v>2025</x:v>
-      </x:c>
-      <x:c r="C111" s="6" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="D111" s="6" t="str">
-        <x:v>Abr</x:v>
-      </x:c>
-      <x:c r="E111" s="6" t="str">
-        <x:v>Fin de semana</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="112">
-      <x:c r="A112" s="6" t="str">
-        <x:v>2025-04-21</x:v>
-      </x:c>
-      <x:c r="B112" s="6" t="n">
-        <x:v>2025</x:v>
-      </x:c>
-      <x:c r="C112" s="6" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="D112" s="6" t="str">
-        <x:v>Abr</x:v>
-      </x:c>
-      <x:c r="E112" s="6" t="str">
-        <x:v>Laboral</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="113">
-      <x:c r="A113" s="6" t="str">
-        <x:v>2025-04-22</x:v>
-      </x:c>
-      <x:c r="B113" s="6" t="n">
-        <x:v>2025</x:v>
-      </x:c>
-      <x:c r="C113" s="6" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="D113" s="6" t="str">
-        <x:v>Abr</x:v>
-      </x:c>
-      <x:c r="E113" s="6" t="str">
-        <x:v>Laboral</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="114">
-      <x:c r="A114" s="6" t="str">
-        <x:v>2025-04-23</x:v>
-      </x:c>
-      <x:c r="B114" s="6" t="n">
-        <x:v>2025</x:v>
-      </x:c>
-      <x:c r="C114" s="6" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="D114" s="6" t="str">
-        <x:v>Abr</x:v>
-      </x:c>
-      <x:c r="E114" s="6" t="str">
-        <x:v>Laboral</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="115">
-      <x:c r="A115" s="6" t="str">
-        <x:v>2025-04-24</x:v>
-      </x:c>
-      <x:c r="B115" s="6" t="n">
-        <x:v>2025</x:v>
-      </x:c>
-      <x:c r="C115" s="6" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="D115" s="6" t="str">
-        <x:v>Abr</x:v>
-      </x:c>
-      <x:c r="E115" s="6" t="str">
-        <x:v>Laboral</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="116">
-      <x:c r="A116" s="6" t="str">
-        <x:v>2025-04-25</x:v>
-      </x:c>
-      <x:c r="B116" s="6" t="n">
-        <x:v>2025</x:v>
-      </x:c>
-      <x:c r="C116" s="6" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="D116" s="6" t="str">
-        <x:v>Abr</x:v>
-      </x:c>
-      <x:c r="E116" s="6" t="str">
-        <x:v>Laboral</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="117">
-      <x:c r="A117" s="6" t="str">
-        <x:v>2025-04-26</x:v>
-      </x:c>
-      <x:c r="B117" s="6" t="n">
-        <x:v>2025</x:v>
-      </x:c>
-      <x:c r="C117" s="6" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="D117" s="6" t="str">
-        <x:v>Abr</x:v>
-      </x:c>
-      <x:c r="E117" s="6" t="str">
-        <x:v>Fin de semana</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="118">
-      <x:c r="A118" s="6" t="str">
-        <x:v>2025-04-27</x:v>
-      </x:c>
-      <x:c r="B118" s="6" t="n">
-        <x:v>2025</x:v>
-      </x:c>
-      <x:c r="C118" s="6" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="D118" s="6" t="str">
-        <x:v>Abr</x:v>
-      </x:c>
-      <x:c r="E118" s="6" t="str">
-        <x:v>Fin de semana</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="119">
-      <x:c r="A119" s="6" t="str">
-        <x:v>2025-04-28</x:v>
-      </x:c>
-      <x:c r="B119" s="6" t="n">
-        <x:v>2025</x:v>
-      </x:c>
-      <x:c r="C119" s="6" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="D119" s="6" t="str">
-        <x:v>Abr</x:v>
-      </x:c>
-      <x:c r="E119" s="6" t="str">
-        <x:v>Laboral</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="120">
-      <x:c r="A120" s="6" t="str">
-        <x:v>2025-04-29</x:v>
-      </x:c>
-      <x:c r="B120" s="6" t="n">
-        <x:v>2025</x:v>
-      </x:c>
-      <x:c r="C120" s="6" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="D120" s="6" t="str">
-        <x:v>Abr</x:v>
-      </x:c>
-      <x:c r="E120" s="6" t="str">
-        <x:v>Laboral</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="121">
-      <x:c r="A121" s="6" t="str">
-        <x:v>2025-04-30</x:v>
-      </x:c>
-      <x:c r="B121" s="6" t="n">
-        <x:v>2025</x:v>
-      </x:c>
-      <x:c r="C121" s="6" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="D121" s="6" t="str">
-        <x:v>Abr</x:v>
-      </x:c>
-      <x:c r="E121" s="6" t="str">
-        <x:v>Laboral</x:v>
-      </x:c>
-    </x:row>
-  </x:sheetData>
-  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R59d9a9a7d93c4aba"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfc23d60676784baa"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>